<commit_message>
uptate Screening summary table
Update Full-text screening (Lack of cohesive contribution)
</commit_message>
<xml_diff>
--- a/Screening_summary_table.xlsx
+++ b/Screening_summary_table.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
   <si>
     <t>Screening summary: reasons for exclusion at each stage</t>
   </si>
@@ -53,15 +53,15 @@
 of Science, Scopus, ScienceDirect, Springer</t>
   </si>
   <si>
+    <t>-</t>
+  </si>
+  <si>
     <t>Pre-screening</t>
   </si>
   <si>
     <t>Duplicate records</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>Title/abstract screening</t>
   </si>
   <si>
@@ -71,7 +71,8 @@
     <t>Relevance (e.g., not physical adversarial attacks)</t>
   </si>
   <si>
-    <t>Full-text screening</t>
+    <t xml:space="preserve">Full-text screening
+</t>
   </si>
   <si>
     <t>Non physical deployment</t>
@@ -83,10 +84,16 @@
     <t>Lack of cohesive contribution</t>
   </si>
   <si>
-    <t>Total</t>
-  </si>
-  <si>
-    <t>All exclusions</t>
+    <t>22. 0%</t>
+  </si>
+  <si>
+    <t>Total exclusions</t>
+  </si>
+  <si>
+    <t>Reports included from database</t>
+  </si>
+  <si>
+    <t>Records included from citation searching</t>
   </si>
   <si>
     <t>ultimately Included</t>
@@ -102,13 +109,20 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FF0F1115"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
@@ -273,7 +287,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="37">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -300,7 +314,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.6"/>
+        <fgColor theme="8" tint="0.8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -491,7 +511,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -549,6 +569,43 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -669,55 +726,52 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -732,74 +786,77 @@
     <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -812,49 +869,64 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="2" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1181,158 +1253,186 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="30" customHeight="1" outlineLevelCol="3"/>
+  <dimension ref="B2:E14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="30" customHeight="1" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="28.875" customWidth="1"/>
-    <col min="2" max="2" width="51.125" customWidth="1"/>
-    <col min="3" max="3" width="40.625" customWidth="1"/>
-    <col min="4" max="4" width="32.625" customWidth="1"/>
+    <col min="2" max="2" width="28.875" customWidth="1"/>
+    <col min="3" max="3" width="51.125" customWidth="1"/>
+    <col min="4" max="4" width="14.125" customWidth="1"/>
+    <col min="5" max="5" width="19.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+    <row r="2" customHeight="1" spans="2:5">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="3"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="3"/>
     </row>
-    <row r="2" ht="32" customHeight="1" spans="1:4">
-      <c r="A2" s="4" t="s">
+    <row r="3" ht="45" customHeight="1" spans="2:5">
+      <c r="B3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E3" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" ht="41" customHeight="1" spans="1:4">
-      <c r="A3" s="5" t="s">
+    <row r="4" ht="41" customHeight="1" spans="2:5">
+      <c r="B4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="C4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="4">
+      <c r="D4" s="4">
         <v>2227</v>
       </c>
-      <c r="D3" s="7"/>
+      <c r="E4" s="7" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="4" ht="32" customHeight="1" spans="1:4">
-      <c r="A4" s="8" t="s">
+    <row r="5" ht="32" customHeight="1" spans="2:5">
+      <c r="B5" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="10">
+        <v>886</v>
+      </c>
+      <c r="E5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="10">
-        <v>886</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>9</v>
-      </c>
     </row>
-    <row r="5" ht="45" customHeight="1" spans="1:4">
-      <c r="A5" s="12" t="s">
+    <row r="6" ht="45" customHeight="1" spans="2:5">
+      <c r="B6" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="C6" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="14">
+      <c r="D6" s="13">
         <v>746</v>
       </c>
-      <c r="D5" s="15">
+      <c r="E6" s="14">
         <v>0.703</v>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1" spans="1:4">
-      <c r="A6" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="13" t="s">
+    <row r="7" ht="32" customHeight="1" spans="2:5">
+      <c r="B7" s="15"/>
+      <c r="C7" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="14">
+      <c r="D7" s="13">
         <v>315</v>
       </c>
-      <c r="D6" s="15">
+      <c r="E7" s="14">
         <v>0.297</v>
       </c>
     </row>
-    <row r="7" ht="32" customHeight="1" spans="1:4">
-      <c r="A7" s="16" t="s">
+    <row r="8" ht="32" customHeight="1" spans="2:5">
+      <c r="B8" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="C8" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="18">
+      <c r="D8" s="18">
         <v>63</v>
       </c>
-      <c r="D7" s="15">
-        <v>0.38</v>
+      <c r="E8" s="14">
+        <v>0.375</v>
       </c>
     </row>
-    <row r="8" ht="32" customHeight="1" spans="1:4">
-      <c r="A8" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="17" t="s">
+    <row r="9" ht="32" customHeight="1" spans="2:5">
+      <c r="B9" s="19"/>
+      <c r="C9" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="18">
+      <c r="D9" s="18">
         <v>68</v>
       </c>
-      <c r="D8" s="15">
-        <v>0.41</v>
+      <c r="E9" s="14">
+        <v>0.405</v>
       </c>
     </row>
-    <row r="9" ht="32" customHeight="1" spans="1:4">
-      <c r="A9" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="17" t="s">
+    <row r="10" ht="32" customHeight="1" spans="2:5">
+      <c r="B10" s="20"/>
+      <c r="C10" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="18">
-        <v>35</v>
-      </c>
-      <c r="D9" s="15">
-        <v>0.211</v>
+      <c r="D10" s="18">
+        <v>37</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="10" ht="32" customHeight="1" spans="1:4">
-      <c r="A10" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" s="6" t="s">
+    <row r="11" customHeight="1" spans="2:5">
+      <c r="B11" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="11">
-        <v>2113</v>
-      </c>
-      <c r="D10" s="11"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="7">
+        <v>2115</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="11" ht="32" customHeight="1" spans="1:4">
-      <c r="A11" s="6" t="s">
+    <row r="12" customHeight="1" spans="2:5">
+      <c r="B12" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11">
+      <c r="C12" s="22"/>
+      <c r="D12" s="7">
+        <v>112</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" customHeight="1" spans="2:5">
+      <c r="B13" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="22"/>
+      <c r="D13" s="7">
+        <v>2</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" customHeight="1" spans="2:5">
+      <c r="B14" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="22"/>
+      <c r="D14" s="23">
         <v>114</v>
       </c>
-      <c r="D11" s="11"/>
+      <c r="E14" s="7" t="s">
+        <v>7</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+  <mergeCells count="7">
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="B8:B10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>